<commit_message>
deploy: main → 31d3fc9204d3347fbc70367ab028bce1080ff5d2
</commit_message>
<xml_diff>
--- a/CodeSystem-assessmentcategory-cs.xlsx
+++ b/CodeSystem-assessmentcategory-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.3.1</t>
+    <t>0.3.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-24T18:50:27+00:00</t>
+    <t>2026-06-25T06:56:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
deploy: main → eb2e893e003118cb342cb00cca1d481e5189fc6f
</commit_message>
<xml_diff>
--- a/CodeSystem-assessmentcategory-cs.xlsx
+++ b/CodeSystem-assessmentcategory-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.3.2</t>
+    <t>0.3.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-25T06:56:03+00:00</t>
+    <t>2026-06-25T07:52:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>